<commit_message>
QC DEPT COA GENERATION VIA PHONE IMPLEMENTED
</commit_message>
<xml_diff>
--- a/backend/app/assets/payroll/AROMAZEN_Bonus_Upload_Template.xlsx
+++ b/backend/app/assets/payroll/AROMAZEN_Bonus_Upload_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus Data" sheetId="1" r:id="R087d649707184c48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rb4b033ace19246a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonus Data" sheetId="1" r:id="R44a0d7de98544044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Re5572866c00d4e8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -378,20 +378,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BonusUploadTable" displayName="BonusUploadTable" ref="A1:L51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="12">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BonusUploadTable" displayName="BonusUploadTable" ref="A1:M51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
     <x:tableColumn id="1" name="Employee Name"/>
     <x:tableColumn id="2" name="Personal Email"/>
     <x:tableColumn id="3" name="Date of Birth"/>
     <x:tableColumn id="4" name="Employee Code"/>
-    <x:tableColumn id="5" name="Date of Joining"/>
-    <x:tableColumn id="6" name="Designation"/>
-    <x:tableColumn id="7" name="UAN"/>
-    <x:tableColumn id="8" name="ESI Number"/>
-    <x:tableColumn id="9" name="Account Number"/>
-    <x:tableColumn id="10" name="Transaction ID"/>
-    <x:tableColumn id="11" name="Payment Date"/>
-    <x:tableColumn id="12" name="Bonus Amount"/>
+    <x:tableColumn id="5" name="Unit"/>
+    <x:tableColumn id="6" name="Date of Joining"/>
+    <x:tableColumn id="7" name="Designation"/>
+    <x:tableColumn id="8" name="UAN"/>
+    <x:tableColumn id="9" name="ESI Number"/>
+    <x:tableColumn id="10" name="Account Number"/>
+    <x:tableColumn id="11" name="Transaction ID"/>
+    <x:tableColumn id="12" name="Payment Date"/>
+    <x:tableColumn id="13" name="Bonus Amount"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -599,14 +600,15 @@
     <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="21" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="21" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -623,27 +625,30 @@
         <x:v>Employee Code</x:v>
       </x:c>
       <x:c r="E1" s="25" t="str">
+        <x:v>Unit</x:v>
+      </x:c>
+      <x:c r="F1" s="25" t="str">
         <x:v>Date of Joining</x:v>
       </x:c>
-      <x:c r="F1" s="25" t="str">
+      <x:c r="G1" s="25" t="str">
         <x:v>Designation</x:v>
       </x:c>
-      <x:c r="G1" s="25" t="str">
+      <x:c r="H1" s="25" t="str">
         <x:v>UAN</x:v>
       </x:c>
-      <x:c r="H1" s="25" t="str">
+      <x:c r="I1" s="25" t="str">
         <x:v>ESI Number</x:v>
       </x:c>
-      <x:c r="I1" s="25" t="str">
+      <x:c r="J1" s="25" t="str">
         <x:v>Account Number</x:v>
       </x:c>
-      <x:c r="J1" s="25" t="str">
+      <x:c r="K1" s="25" t="str">
         <x:v>Transaction ID</x:v>
       </x:c>
-      <x:c r="K1" s="25" t="str">
+      <x:c r="L1" s="25" t="str">
         <x:v>Payment Date</x:v>
       </x:c>
-      <x:c r="L1" s="26" t="str">
+      <x:c r="M1" s="26" t="str">
         <x:v>Bonus Amount</x:v>
       </x:c>
     </x:row>
@@ -660,28 +665,31 @@
       <x:c r="D2" s="28" t="str">
         <x:v>EMP001</x:v>
       </x:c>
-      <x:c r="E2" s="29" t="n">
+      <x:c r="E2" s="28" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="29" t="n">
         <x:v>44571</x:v>
       </x:c>
-      <x:c r="F2" s="28" t="str">
+      <x:c r="G2" s="28" t="str">
         <x:v>Executive</x:v>
       </x:c>
-      <x:c r="G2" s="30" t="str">
+      <x:c r="H2" s="30" t="str">
         <x:v>UAN-100000000000</x:v>
       </x:c>
-      <x:c r="H2" s="30" t="str">
+      <x:c r="I2" s="30" t="str">
         <x:v>ESI-1234567890</x:v>
       </x:c>
-      <x:c r="I2" s="30" t="str">
+      <x:c r="J2" s="30" t="str">
         <x:v>AC-123456789012</x:v>
       </x:c>
-      <x:c r="J2" s="30" t="str">
+      <x:c r="K2" s="30" t="str">
         <x:v>TXN-2026-001</x:v>
       </x:c>
-      <x:c r="K2" s="29" t="n">
+      <x:c r="L2" s="29" t="n">
         <x:v>46280</x:v>
       </x:c>
-      <x:c r="L2" s="31" t="n">
+      <x:c r="M2" s="31" t="n">
         <x:v>25000</x:v>
       </x:c>
     </x:row>
@@ -690,691 +698,745 @@
       <x:c r="B3" s="33"/>
       <x:c r="C3" s="34"/>
       <x:c r="D3" s="33"/>
-      <x:c r="E3" s="34"/>
-      <x:c r="F3" s="33"/>
-      <x:c r="G3" s="35"/>
+      <x:c r="E3" s="33"/>
+      <x:c r="F3" s="34"/>
+      <x:c r="G3" s="33"/>
       <x:c r="H3" s="35"/>
       <x:c r="I3" s="35"/>
       <x:c r="J3" s="35"/>
-      <x:c r="K3" s="34"/>
-      <x:c r="L3" s="36"/>
+      <x:c r="K3" s="35"/>
+      <x:c r="L3" s="34"/>
+      <x:c r="M3" s="36"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="32"/>
       <x:c r="B4" s="33"/>
       <x:c r="C4" s="34"/>
       <x:c r="D4" s="33"/>
-      <x:c r="E4" s="34"/>
-      <x:c r="F4" s="33"/>
-      <x:c r="G4" s="35"/>
+      <x:c r="E4" s="33"/>
+      <x:c r="F4" s="34"/>
+      <x:c r="G4" s="33"/>
       <x:c r="H4" s="35"/>
       <x:c r="I4" s="35"/>
       <x:c r="J4" s="35"/>
-      <x:c r="K4" s="34"/>
-      <x:c r="L4" s="36"/>
+      <x:c r="K4" s="35"/>
+      <x:c r="L4" s="34"/>
+      <x:c r="M4" s="36"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="32"/>
       <x:c r="B5" s="33"/>
       <x:c r="C5" s="34"/>
       <x:c r="D5" s="33"/>
-      <x:c r="E5" s="34"/>
-      <x:c r="F5" s="33"/>
-      <x:c r="G5" s="35"/>
+      <x:c r="E5" s="33"/>
+      <x:c r="F5" s="34"/>
+      <x:c r="G5" s="33"/>
       <x:c r="H5" s="35"/>
       <x:c r="I5" s="35"/>
       <x:c r="J5" s="35"/>
-      <x:c r="K5" s="34"/>
-      <x:c r="L5" s="36"/>
+      <x:c r="K5" s="35"/>
+      <x:c r="L5" s="34"/>
+      <x:c r="M5" s="36"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="32"/>
       <x:c r="B6" s="33"/>
       <x:c r="C6" s="34"/>
       <x:c r="D6" s="33"/>
-      <x:c r="E6" s="34"/>
-      <x:c r="F6" s="33"/>
-      <x:c r="G6" s="35"/>
+      <x:c r="E6" s="33"/>
+      <x:c r="F6" s="34"/>
+      <x:c r="G6" s="33"/>
       <x:c r="H6" s="35"/>
       <x:c r="I6" s="35"/>
       <x:c r="J6" s="35"/>
-      <x:c r="K6" s="34"/>
-      <x:c r="L6" s="36"/>
+      <x:c r="K6" s="35"/>
+      <x:c r="L6" s="34"/>
+      <x:c r="M6" s="36"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="32"/>
       <x:c r="B7" s="33"/>
       <x:c r="C7" s="34"/>
       <x:c r="D7" s="33"/>
-      <x:c r="E7" s="34"/>
-      <x:c r="F7" s="33"/>
-      <x:c r="G7" s="35"/>
+      <x:c r="E7" s="33"/>
+      <x:c r="F7" s="34"/>
+      <x:c r="G7" s="33"/>
       <x:c r="H7" s="35"/>
       <x:c r="I7" s="35"/>
       <x:c r="J7" s="35"/>
-      <x:c r="K7" s="34"/>
-      <x:c r="L7" s="36"/>
+      <x:c r="K7" s="35"/>
+      <x:c r="L7" s="34"/>
+      <x:c r="M7" s="36"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="32"/>
       <x:c r="B8" s="33"/>
       <x:c r="C8" s="34"/>
       <x:c r="D8" s="33"/>
-      <x:c r="E8" s="34"/>
-      <x:c r="F8" s="33"/>
-      <x:c r="G8" s="35"/>
+      <x:c r="E8" s="33"/>
+      <x:c r="F8" s="34"/>
+      <x:c r="G8" s="33"/>
       <x:c r="H8" s="35"/>
       <x:c r="I8" s="35"/>
       <x:c r="J8" s="35"/>
-      <x:c r="K8" s="34"/>
-      <x:c r="L8" s="36"/>
+      <x:c r="K8" s="35"/>
+      <x:c r="L8" s="34"/>
+      <x:c r="M8" s="36"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="32"/>
       <x:c r="B9" s="33"/>
       <x:c r="C9" s="34"/>
       <x:c r="D9" s="33"/>
-      <x:c r="E9" s="34"/>
-      <x:c r="F9" s="33"/>
-      <x:c r="G9" s="35"/>
+      <x:c r="E9" s="33"/>
+      <x:c r="F9" s="34"/>
+      <x:c r="G9" s="33"/>
       <x:c r="H9" s="35"/>
       <x:c r="I9" s="35"/>
       <x:c r="J9" s="35"/>
-      <x:c r="K9" s="34"/>
-      <x:c r="L9" s="36"/>
+      <x:c r="K9" s="35"/>
+      <x:c r="L9" s="34"/>
+      <x:c r="M9" s="36"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="32"/>
       <x:c r="B10" s="33"/>
       <x:c r="C10" s="34"/>
       <x:c r="D10" s="33"/>
-      <x:c r="E10" s="34"/>
-      <x:c r="F10" s="33"/>
-      <x:c r="G10" s="35"/>
+      <x:c r="E10" s="33"/>
+      <x:c r="F10" s="34"/>
+      <x:c r="G10" s="33"/>
       <x:c r="H10" s="35"/>
       <x:c r="I10" s="35"/>
       <x:c r="J10" s="35"/>
-      <x:c r="K10" s="34"/>
-      <x:c r="L10" s="36"/>
+      <x:c r="K10" s="35"/>
+      <x:c r="L10" s="34"/>
+      <x:c r="M10" s="36"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="32"/>
       <x:c r="B11" s="33"/>
       <x:c r="C11" s="34"/>
       <x:c r="D11" s="33"/>
-      <x:c r="E11" s="34"/>
-      <x:c r="F11" s="33"/>
-      <x:c r="G11" s="35"/>
+      <x:c r="E11" s="33"/>
+      <x:c r="F11" s="34"/>
+      <x:c r="G11" s="33"/>
       <x:c r="H11" s="35"/>
       <x:c r="I11" s="35"/>
       <x:c r="J11" s="35"/>
-      <x:c r="K11" s="34"/>
-      <x:c r="L11" s="36"/>
+      <x:c r="K11" s="35"/>
+      <x:c r="L11" s="34"/>
+      <x:c r="M11" s="36"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="32"/>
       <x:c r="B12" s="33"/>
       <x:c r="C12" s="34"/>
       <x:c r="D12" s="33"/>
-      <x:c r="E12" s="34"/>
-      <x:c r="F12" s="33"/>
-      <x:c r="G12" s="35"/>
+      <x:c r="E12" s="33"/>
+      <x:c r="F12" s="34"/>
+      <x:c r="G12" s="33"/>
       <x:c r="H12" s="35"/>
       <x:c r="I12" s="35"/>
       <x:c r="J12" s="35"/>
-      <x:c r="K12" s="34"/>
-      <x:c r="L12" s="36"/>
+      <x:c r="K12" s="35"/>
+      <x:c r="L12" s="34"/>
+      <x:c r="M12" s="36"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="32"/>
       <x:c r="B13" s="33"/>
       <x:c r="C13" s="34"/>
       <x:c r="D13" s="33"/>
-      <x:c r="E13" s="34"/>
-      <x:c r="F13" s="33"/>
-      <x:c r="G13" s="35"/>
+      <x:c r="E13" s="33"/>
+      <x:c r="F13" s="34"/>
+      <x:c r="G13" s="33"/>
       <x:c r="H13" s="35"/>
       <x:c r="I13" s="35"/>
       <x:c r="J13" s="35"/>
-      <x:c r="K13" s="34"/>
-      <x:c r="L13" s="36"/>
+      <x:c r="K13" s="35"/>
+      <x:c r="L13" s="34"/>
+      <x:c r="M13" s="36"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="32"/>
       <x:c r="B14" s="33"/>
       <x:c r="C14" s="34"/>
       <x:c r="D14" s="33"/>
-      <x:c r="E14" s="34"/>
-      <x:c r="F14" s="33"/>
-      <x:c r="G14" s="35"/>
+      <x:c r="E14" s="33"/>
+      <x:c r="F14" s="34"/>
+      <x:c r="G14" s="33"/>
       <x:c r="H14" s="35"/>
       <x:c r="I14" s="35"/>
       <x:c r="J14" s="35"/>
-      <x:c r="K14" s="34"/>
-      <x:c r="L14" s="36"/>
+      <x:c r="K14" s="35"/>
+      <x:c r="L14" s="34"/>
+      <x:c r="M14" s="36"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="32"/>
       <x:c r="B15" s="33"/>
       <x:c r="C15" s="34"/>
       <x:c r="D15" s="33"/>
-      <x:c r="E15" s="34"/>
-      <x:c r="F15" s="33"/>
-      <x:c r="G15" s="35"/>
+      <x:c r="E15" s="33"/>
+      <x:c r="F15" s="34"/>
+      <x:c r="G15" s="33"/>
       <x:c r="H15" s="35"/>
       <x:c r="I15" s="35"/>
       <x:c r="J15" s="35"/>
-      <x:c r="K15" s="34"/>
-      <x:c r="L15" s="36"/>
+      <x:c r="K15" s="35"/>
+      <x:c r="L15" s="34"/>
+      <x:c r="M15" s="36"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32"/>
       <x:c r="B16" s="33"/>
       <x:c r="C16" s="34"/>
       <x:c r="D16" s="33"/>
-      <x:c r="E16" s="34"/>
-      <x:c r="F16" s="33"/>
-      <x:c r="G16" s="35"/>
+      <x:c r="E16" s="33"/>
+      <x:c r="F16" s="34"/>
+      <x:c r="G16" s="33"/>
       <x:c r="H16" s="35"/>
       <x:c r="I16" s="35"/>
       <x:c r="J16" s="35"/>
-      <x:c r="K16" s="34"/>
-      <x:c r="L16" s="36"/>
+      <x:c r="K16" s="35"/>
+      <x:c r="L16" s="34"/>
+      <x:c r="M16" s="36"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="32"/>
       <x:c r="B17" s="33"/>
       <x:c r="C17" s="34"/>
       <x:c r="D17" s="33"/>
-      <x:c r="E17" s="34"/>
-      <x:c r="F17" s="33"/>
-      <x:c r="G17" s="35"/>
+      <x:c r="E17" s="33"/>
+      <x:c r="F17" s="34"/>
+      <x:c r="G17" s="33"/>
       <x:c r="H17" s="35"/>
       <x:c r="I17" s="35"/>
       <x:c r="J17" s="35"/>
-      <x:c r="K17" s="34"/>
-      <x:c r="L17" s="36"/>
+      <x:c r="K17" s="35"/>
+      <x:c r="L17" s="34"/>
+      <x:c r="M17" s="36"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="32"/>
       <x:c r="B18" s="33"/>
       <x:c r="C18" s="34"/>
       <x:c r="D18" s="33"/>
-      <x:c r="E18" s="34"/>
-      <x:c r="F18" s="33"/>
-      <x:c r="G18" s="35"/>
+      <x:c r="E18" s="33"/>
+      <x:c r="F18" s="34"/>
+      <x:c r="G18" s="33"/>
       <x:c r="H18" s="35"/>
       <x:c r="I18" s="35"/>
       <x:c r="J18" s="35"/>
-      <x:c r="K18" s="34"/>
-      <x:c r="L18" s="36"/>
+      <x:c r="K18" s="35"/>
+      <x:c r="L18" s="34"/>
+      <x:c r="M18" s="36"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="32"/>
       <x:c r="B19" s="33"/>
       <x:c r="C19" s="34"/>
       <x:c r="D19" s="33"/>
-      <x:c r="E19" s="34"/>
-      <x:c r="F19" s="33"/>
-      <x:c r="G19" s="35"/>
+      <x:c r="E19" s="33"/>
+      <x:c r="F19" s="34"/>
+      <x:c r="G19" s="33"/>
       <x:c r="H19" s="35"/>
       <x:c r="I19" s="35"/>
       <x:c r="J19" s="35"/>
-      <x:c r="K19" s="34"/>
-      <x:c r="L19" s="36"/>
+      <x:c r="K19" s="35"/>
+      <x:c r="L19" s="34"/>
+      <x:c r="M19" s="36"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="32"/>
       <x:c r="B20" s="33"/>
       <x:c r="C20" s="34"/>
       <x:c r="D20" s="33"/>
-      <x:c r="E20" s="34"/>
-      <x:c r="F20" s="33"/>
-      <x:c r="G20" s="35"/>
+      <x:c r="E20" s="33"/>
+      <x:c r="F20" s="34"/>
+      <x:c r="G20" s="33"/>
       <x:c r="H20" s="35"/>
       <x:c r="I20" s="35"/>
       <x:c r="J20" s="35"/>
-      <x:c r="K20" s="34"/>
-      <x:c r="L20" s="36"/>
+      <x:c r="K20" s="35"/>
+      <x:c r="L20" s="34"/>
+      <x:c r="M20" s="36"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="32"/>
       <x:c r="B21" s="33"/>
       <x:c r="C21" s="34"/>
       <x:c r="D21" s="33"/>
-      <x:c r="E21" s="34"/>
-      <x:c r="F21" s="33"/>
-      <x:c r="G21" s="35"/>
+      <x:c r="E21" s="33"/>
+      <x:c r="F21" s="34"/>
+      <x:c r="G21" s="33"/>
       <x:c r="H21" s="35"/>
       <x:c r="I21" s="35"/>
       <x:c r="J21" s="35"/>
-      <x:c r="K21" s="34"/>
-      <x:c r="L21" s="36"/>
+      <x:c r="K21" s="35"/>
+      <x:c r="L21" s="34"/>
+      <x:c r="M21" s="36"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="32"/>
       <x:c r="B22" s="33"/>
       <x:c r="C22" s="34"/>
       <x:c r="D22" s="33"/>
-      <x:c r="E22" s="34"/>
-      <x:c r="F22" s="33"/>
-      <x:c r="G22" s="35"/>
+      <x:c r="E22" s="33"/>
+      <x:c r="F22" s="34"/>
+      <x:c r="G22" s="33"/>
       <x:c r="H22" s="35"/>
       <x:c r="I22" s="35"/>
       <x:c r="J22" s="35"/>
-      <x:c r="K22" s="34"/>
-      <x:c r="L22" s="36"/>
+      <x:c r="K22" s="35"/>
+      <x:c r="L22" s="34"/>
+      <x:c r="M22" s="36"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="32"/>
       <x:c r="B23" s="33"/>
       <x:c r="C23" s="34"/>
       <x:c r="D23" s="33"/>
-      <x:c r="E23" s="34"/>
-      <x:c r="F23" s="33"/>
-      <x:c r="G23" s="35"/>
+      <x:c r="E23" s="33"/>
+      <x:c r="F23" s="34"/>
+      <x:c r="G23" s="33"/>
       <x:c r="H23" s="35"/>
       <x:c r="I23" s="35"/>
       <x:c r="J23" s="35"/>
-      <x:c r="K23" s="34"/>
-      <x:c r="L23" s="36"/>
+      <x:c r="K23" s="35"/>
+      <x:c r="L23" s="34"/>
+      <x:c r="M23" s="36"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="32"/>
       <x:c r="B24" s="33"/>
       <x:c r="C24" s="34"/>
       <x:c r="D24" s="33"/>
-      <x:c r="E24" s="34"/>
-      <x:c r="F24" s="33"/>
-      <x:c r="G24" s="35"/>
+      <x:c r="E24" s="33"/>
+      <x:c r="F24" s="34"/>
+      <x:c r="G24" s="33"/>
       <x:c r="H24" s="35"/>
       <x:c r="I24" s="35"/>
       <x:c r="J24" s="35"/>
-      <x:c r="K24" s="34"/>
-      <x:c r="L24" s="36"/>
+      <x:c r="K24" s="35"/>
+      <x:c r="L24" s="34"/>
+      <x:c r="M24" s="36"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="32"/>
       <x:c r="B25" s="33"/>
       <x:c r="C25" s="34"/>
       <x:c r="D25" s="33"/>
-      <x:c r="E25" s="34"/>
-      <x:c r="F25" s="33"/>
-      <x:c r="G25" s="35"/>
+      <x:c r="E25" s="33"/>
+      <x:c r="F25" s="34"/>
+      <x:c r="G25" s="33"/>
       <x:c r="H25" s="35"/>
       <x:c r="I25" s="35"/>
       <x:c r="J25" s="35"/>
-      <x:c r="K25" s="34"/>
-      <x:c r="L25" s="36"/>
+      <x:c r="K25" s="35"/>
+      <x:c r="L25" s="34"/>
+      <x:c r="M25" s="36"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="32"/>
       <x:c r="B26" s="33"/>
       <x:c r="C26" s="34"/>
       <x:c r="D26" s="33"/>
-      <x:c r="E26" s="34"/>
-      <x:c r="F26" s="33"/>
-      <x:c r="G26" s="35"/>
+      <x:c r="E26" s="33"/>
+      <x:c r="F26" s="34"/>
+      <x:c r="G26" s="33"/>
       <x:c r="H26" s="35"/>
       <x:c r="I26" s="35"/>
       <x:c r="J26" s="35"/>
-      <x:c r="K26" s="34"/>
-      <x:c r="L26" s="36"/>
+      <x:c r="K26" s="35"/>
+      <x:c r="L26" s="34"/>
+      <x:c r="M26" s="36"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="32"/>
       <x:c r="B27" s="33"/>
       <x:c r="C27" s="34"/>
       <x:c r="D27" s="33"/>
-      <x:c r="E27" s="34"/>
-      <x:c r="F27" s="33"/>
-      <x:c r="G27" s="35"/>
+      <x:c r="E27" s="33"/>
+      <x:c r="F27" s="34"/>
+      <x:c r="G27" s="33"/>
       <x:c r="H27" s="35"/>
       <x:c r="I27" s="35"/>
       <x:c r="J27" s="35"/>
-      <x:c r="K27" s="34"/>
-      <x:c r="L27" s="36"/>
+      <x:c r="K27" s="35"/>
+      <x:c r="L27" s="34"/>
+      <x:c r="M27" s="36"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="32"/>
       <x:c r="B28" s="33"/>
       <x:c r="C28" s="34"/>
       <x:c r="D28" s="33"/>
-      <x:c r="E28" s="34"/>
-      <x:c r="F28" s="33"/>
-      <x:c r="G28" s="35"/>
+      <x:c r="E28" s="33"/>
+      <x:c r="F28" s="34"/>
+      <x:c r="G28" s="33"/>
       <x:c r="H28" s="35"/>
       <x:c r="I28" s="35"/>
       <x:c r="J28" s="35"/>
-      <x:c r="K28" s="34"/>
-      <x:c r="L28" s="36"/>
+      <x:c r="K28" s="35"/>
+      <x:c r="L28" s="34"/>
+      <x:c r="M28" s="36"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="32"/>
       <x:c r="B29" s="33"/>
       <x:c r="C29" s="34"/>
       <x:c r="D29" s="33"/>
-      <x:c r="E29" s="34"/>
-      <x:c r="F29" s="33"/>
-      <x:c r="G29" s="35"/>
+      <x:c r="E29" s="33"/>
+      <x:c r="F29" s="34"/>
+      <x:c r="G29" s="33"/>
       <x:c r="H29" s="35"/>
       <x:c r="I29" s="35"/>
       <x:c r="J29" s="35"/>
-      <x:c r="K29" s="34"/>
-      <x:c r="L29" s="36"/>
+      <x:c r="K29" s="35"/>
+      <x:c r="L29" s="34"/>
+      <x:c r="M29" s="36"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="32"/>
       <x:c r="B30" s="33"/>
       <x:c r="C30" s="34"/>
       <x:c r="D30" s="33"/>
-      <x:c r="E30" s="34"/>
-      <x:c r="F30" s="33"/>
-      <x:c r="G30" s="35"/>
+      <x:c r="E30" s="33"/>
+      <x:c r="F30" s="34"/>
+      <x:c r="G30" s="33"/>
       <x:c r="H30" s="35"/>
       <x:c r="I30" s="35"/>
       <x:c r="J30" s="35"/>
-      <x:c r="K30" s="34"/>
-      <x:c r="L30" s="36"/>
+      <x:c r="K30" s="35"/>
+      <x:c r="L30" s="34"/>
+      <x:c r="M30" s="36"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="32"/>
       <x:c r="B31" s="33"/>
       <x:c r="C31" s="34"/>
       <x:c r="D31" s="33"/>
-      <x:c r="E31" s="34"/>
-      <x:c r="F31" s="33"/>
-      <x:c r="G31" s="35"/>
+      <x:c r="E31" s="33"/>
+      <x:c r="F31" s="34"/>
+      <x:c r="G31" s="33"/>
       <x:c r="H31" s="35"/>
       <x:c r="I31" s="35"/>
       <x:c r="J31" s="35"/>
-      <x:c r="K31" s="34"/>
-      <x:c r="L31" s="36"/>
+      <x:c r="K31" s="35"/>
+      <x:c r="L31" s="34"/>
+      <x:c r="M31" s="36"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="32"/>
       <x:c r="B32" s="33"/>
       <x:c r="C32" s="34"/>
       <x:c r="D32" s="33"/>
-      <x:c r="E32" s="34"/>
-      <x:c r="F32" s="33"/>
-      <x:c r="G32" s="35"/>
+      <x:c r="E32" s="33"/>
+      <x:c r="F32" s="34"/>
+      <x:c r="G32" s="33"/>
       <x:c r="H32" s="35"/>
       <x:c r="I32" s="35"/>
       <x:c r="J32" s="35"/>
-      <x:c r="K32" s="34"/>
-      <x:c r="L32" s="36"/>
+      <x:c r="K32" s="35"/>
+      <x:c r="L32" s="34"/>
+      <x:c r="M32" s="36"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="32"/>
       <x:c r="B33" s="33"/>
       <x:c r="C33" s="34"/>
       <x:c r="D33" s="33"/>
-      <x:c r="E33" s="34"/>
-      <x:c r="F33" s="33"/>
-      <x:c r="G33" s="35"/>
+      <x:c r="E33" s="33"/>
+      <x:c r="F33" s="34"/>
+      <x:c r="G33" s="33"/>
       <x:c r="H33" s="35"/>
       <x:c r="I33" s="35"/>
       <x:c r="J33" s="35"/>
-      <x:c r="K33" s="34"/>
-      <x:c r="L33" s="36"/>
+      <x:c r="K33" s="35"/>
+      <x:c r="L33" s="34"/>
+      <x:c r="M33" s="36"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="32"/>
       <x:c r="B34" s="33"/>
       <x:c r="C34" s="34"/>
       <x:c r="D34" s="33"/>
-      <x:c r="E34" s="34"/>
-      <x:c r="F34" s="33"/>
-      <x:c r="G34" s="35"/>
+      <x:c r="E34" s="33"/>
+      <x:c r="F34" s="34"/>
+      <x:c r="G34" s="33"/>
       <x:c r="H34" s="35"/>
       <x:c r="I34" s="35"/>
       <x:c r="J34" s="35"/>
-      <x:c r="K34" s="34"/>
-      <x:c r="L34" s="36"/>
+      <x:c r="K34" s="35"/>
+      <x:c r="L34" s="34"/>
+      <x:c r="M34" s="36"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="32"/>
       <x:c r="B35" s="33"/>
       <x:c r="C35" s="34"/>
       <x:c r="D35" s="33"/>
-      <x:c r="E35" s="34"/>
-      <x:c r="F35" s="33"/>
-      <x:c r="G35" s="35"/>
+      <x:c r="E35" s="33"/>
+      <x:c r="F35" s="34"/>
+      <x:c r="G35" s="33"/>
       <x:c r="H35" s="35"/>
       <x:c r="I35" s="35"/>
       <x:c r="J35" s="35"/>
-      <x:c r="K35" s="34"/>
-      <x:c r="L35" s="36"/>
+      <x:c r="K35" s="35"/>
+      <x:c r="L35" s="34"/>
+      <x:c r="M35" s="36"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="32"/>
       <x:c r="B36" s="33"/>
       <x:c r="C36" s="34"/>
       <x:c r="D36" s="33"/>
-      <x:c r="E36" s="34"/>
-      <x:c r="F36" s="33"/>
-      <x:c r="G36" s="35"/>
+      <x:c r="E36" s="33"/>
+      <x:c r="F36" s="34"/>
+      <x:c r="G36" s="33"/>
       <x:c r="H36" s="35"/>
       <x:c r="I36" s="35"/>
       <x:c r="J36" s="35"/>
-      <x:c r="K36" s="34"/>
-      <x:c r="L36" s="36"/>
+      <x:c r="K36" s="35"/>
+      <x:c r="L36" s="34"/>
+      <x:c r="M36" s="36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="32"/>
       <x:c r="B37" s="33"/>
       <x:c r="C37" s="34"/>
       <x:c r="D37" s="33"/>
-      <x:c r="E37" s="34"/>
-      <x:c r="F37" s="33"/>
-      <x:c r="G37" s="35"/>
+      <x:c r="E37" s="33"/>
+      <x:c r="F37" s="34"/>
+      <x:c r="G37" s="33"/>
       <x:c r="H37" s="35"/>
       <x:c r="I37" s="35"/>
       <x:c r="J37" s="35"/>
-      <x:c r="K37" s="34"/>
-      <x:c r="L37" s="36"/>
+      <x:c r="K37" s="35"/>
+      <x:c r="L37" s="34"/>
+      <x:c r="M37" s="36"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="32"/>
       <x:c r="B38" s="33"/>
       <x:c r="C38" s="34"/>
       <x:c r="D38" s="33"/>
-      <x:c r="E38" s="34"/>
-      <x:c r="F38" s="33"/>
-      <x:c r="G38" s="35"/>
+      <x:c r="E38" s="33"/>
+      <x:c r="F38" s="34"/>
+      <x:c r="G38" s="33"/>
       <x:c r="H38" s="35"/>
       <x:c r="I38" s="35"/>
       <x:c r="J38" s="35"/>
-      <x:c r="K38" s="34"/>
-      <x:c r="L38" s="36"/>
+      <x:c r="K38" s="35"/>
+      <x:c r="L38" s="34"/>
+      <x:c r="M38" s="36"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="32"/>
       <x:c r="B39" s="33"/>
       <x:c r="C39" s="34"/>
       <x:c r="D39" s="33"/>
-      <x:c r="E39" s="34"/>
-      <x:c r="F39" s="33"/>
-      <x:c r="G39" s="35"/>
+      <x:c r="E39" s="33"/>
+      <x:c r="F39" s="34"/>
+      <x:c r="G39" s="33"/>
       <x:c r="H39" s="35"/>
       <x:c r="I39" s="35"/>
       <x:c r="J39" s="35"/>
-      <x:c r="K39" s="34"/>
-      <x:c r="L39" s="36"/>
+      <x:c r="K39" s="35"/>
+      <x:c r="L39" s="34"/>
+      <x:c r="M39" s="36"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="32"/>
       <x:c r="B40" s="33"/>
       <x:c r="C40" s="34"/>
       <x:c r="D40" s="33"/>
-      <x:c r="E40" s="34"/>
-      <x:c r="F40" s="33"/>
-      <x:c r="G40" s="35"/>
+      <x:c r="E40" s="33"/>
+      <x:c r="F40" s="34"/>
+      <x:c r="G40" s="33"/>
       <x:c r="H40" s="35"/>
       <x:c r="I40" s="35"/>
       <x:c r="J40" s="35"/>
-      <x:c r="K40" s="34"/>
-      <x:c r="L40" s="36"/>
+      <x:c r="K40" s="35"/>
+      <x:c r="L40" s="34"/>
+      <x:c r="M40" s="36"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="32"/>
       <x:c r="B41" s="33"/>
       <x:c r="C41" s="34"/>
       <x:c r="D41" s="33"/>
-      <x:c r="E41" s="34"/>
-      <x:c r="F41" s="33"/>
-      <x:c r="G41" s="35"/>
+      <x:c r="E41" s="33"/>
+      <x:c r="F41" s="34"/>
+      <x:c r="G41" s="33"/>
       <x:c r="H41" s="35"/>
       <x:c r="I41" s="35"/>
       <x:c r="J41" s="35"/>
-      <x:c r="K41" s="34"/>
-      <x:c r="L41" s="36"/>
+      <x:c r="K41" s="35"/>
+      <x:c r="L41" s="34"/>
+      <x:c r="M41" s="36"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="32"/>
       <x:c r="B42" s="33"/>
       <x:c r="C42" s="34"/>
       <x:c r="D42" s="33"/>
-      <x:c r="E42" s="34"/>
-      <x:c r="F42" s="33"/>
-      <x:c r="G42" s="35"/>
+      <x:c r="E42" s="33"/>
+      <x:c r="F42" s="34"/>
+      <x:c r="G42" s="33"/>
       <x:c r="H42" s="35"/>
       <x:c r="I42" s="35"/>
       <x:c r="J42" s="35"/>
-      <x:c r="K42" s="34"/>
-      <x:c r="L42" s="36"/>
+      <x:c r="K42" s="35"/>
+      <x:c r="L42" s="34"/>
+      <x:c r="M42" s="36"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="32"/>
       <x:c r="B43" s="33"/>
       <x:c r="C43" s="34"/>
       <x:c r="D43" s="33"/>
-      <x:c r="E43" s="34"/>
-      <x:c r="F43" s="33"/>
-      <x:c r="G43" s="35"/>
+      <x:c r="E43" s="33"/>
+      <x:c r="F43" s="34"/>
+      <x:c r="G43" s="33"/>
       <x:c r="H43" s="35"/>
       <x:c r="I43" s="35"/>
       <x:c r="J43" s="35"/>
-      <x:c r="K43" s="34"/>
-      <x:c r="L43" s="36"/>
+      <x:c r="K43" s="35"/>
+      <x:c r="L43" s="34"/>
+      <x:c r="M43" s="36"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="32"/>
       <x:c r="B44" s="33"/>
       <x:c r="C44" s="34"/>
       <x:c r="D44" s="33"/>
-      <x:c r="E44" s="34"/>
-      <x:c r="F44" s="33"/>
-      <x:c r="G44" s="35"/>
+      <x:c r="E44" s="33"/>
+      <x:c r="F44" s="34"/>
+      <x:c r="G44" s="33"/>
       <x:c r="H44" s="35"/>
       <x:c r="I44" s="35"/>
       <x:c r="J44" s="35"/>
-      <x:c r="K44" s="34"/>
-      <x:c r="L44" s="36"/>
+      <x:c r="K44" s="35"/>
+      <x:c r="L44" s="34"/>
+      <x:c r="M44" s="36"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="32"/>
       <x:c r="B45" s="33"/>
       <x:c r="C45" s="34"/>
       <x:c r="D45" s="33"/>
-      <x:c r="E45" s="34"/>
-      <x:c r="F45" s="33"/>
-      <x:c r="G45" s="35"/>
+      <x:c r="E45" s="33"/>
+      <x:c r="F45" s="34"/>
+      <x:c r="G45" s="33"/>
       <x:c r="H45" s="35"/>
       <x:c r="I45" s="35"/>
       <x:c r="J45" s="35"/>
-      <x:c r="K45" s="34"/>
-      <x:c r="L45" s="36"/>
+      <x:c r="K45" s="35"/>
+      <x:c r="L45" s="34"/>
+      <x:c r="M45" s="36"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="32"/>
       <x:c r="B46" s="33"/>
       <x:c r="C46" s="34"/>
       <x:c r="D46" s="33"/>
-      <x:c r="E46" s="34"/>
-      <x:c r="F46" s="33"/>
-      <x:c r="G46" s="35"/>
+      <x:c r="E46" s="33"/>
+      <x:c r="F46" s="34"/>
+      <x:c r="G46" s="33"/>
       <x:c r="H46" s="35"/>
       <x:c r="I46" s="35"/>
       <x:c r="J46" s="35"/>
-      <x:c r="K46" s="34"/>
-      <x:c r="L46" s="36"/>
+      <x:c r="K46" s="35"/>
+      <x:c r="L46" s="34"/>
+      <x:c r="M46" s="36"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="32"/>
       <x:c r="B47" s="33"/>
       <x:c r="C47" s="34"/>
       <x:c r="D47" s="33"/>
-      <x:c r="E47" s="34"/>
-      <x:c r="F47" s="33"/>
-      <x:c r="G47" s="35"/>
+      <x:c r="E47" s="33"/>
+      <x:c r="F47" s="34"/>
+      <x:c r="G47" s="33"/>
       <x:c r="H47" s="35"/>
       <x:c r="I47" s="35"/>
       <x:c r="J47" s="35"/>
-      <x:c r="K47" s="34"/>
-      <x:c r="L47" s="36"/>
+      <x:c r="K47" s="35"/>
+      <x:c r="L47" s="34"/>
+      <x:c r="M47" s="36"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="32"/>
       <x:c r="B48" s="33"/>
       <x:c r="C48" s="34"/>
       <x:c r="D48" s="33"/>
-      <x:c r="E48" s="34"/>
-      <x:c r="F48" s="33"/>
-      <x:c r="G48" s="35"/>
+      <x:c r="E48" s="33"/>
+      <x:c r="F48" s="34"/>
+      <x:c r="G48" s="33"/>
       <x:c r="H48" s="35"/>
       <x:c r="I48" s="35"/>
       <x:c r="J48" s="35"/>
-      <x:c r="K48" s="34"/>
-      <x:c r="L48" s="36"/>
+      <x:c r="K48" s="35"/>
+      <x:c r="L48" s="34"/>
+      <x:c r="M48" s="36"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="32"/>
       <x:c r="B49" s="33"/>
       <x:c r="C49" s="34"/>
       <x:c r="D49" s="33"/>
-      <x:c r="E49" s="34"/>
-      <x:c r="F49" s="33"/>
-      <x:c r="G49" s="35"/>
+      <x:c r="E49" s="33"/>
+      <x:c r="F49" s="34"/>
+      <x:c r="G49" s="33"/>
       <x:c r="H49" s="35"/>
       <x:c r="I49" s="35"/>
       <x:c r="J49" s="35"/>
-      <x:c r="K49" s="34"/>
-      <x:c r="L49" s="36"/>
+      <x:c r="K49" s="35"/>
+      <x:c r="L49" s="34"/>
+      <x:c r="M49" s="36"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="32"/>
       <x:c r="B50" s="33"/>
       <x:c r="C50" s="34"/>
       <x:c r="D50" s="33"/>
-      <x:c r="E50" s="34"/>
-      <x:c r="F50" s="33"/>
-      <x:c r="G50" s="35"/>
+      <x:c r="E50" s="33"/>
+      <x:c r="F50" s="34"/>
+      <x:c r="G50" s="33"/>
       <x:c r="H50" s="35"/>
       <x:c r="I50" s="35"/>
       <x:c r="J50" s="35"/>
-      <x:c r="K50" s="34"/>
-      <x:c r="L50" s="36"/>
+      <x:c r="K50" s="35"/>
+      <x:c r="L50" s="34"/>
+      <x:c r="M50" s="36"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="37"/>
       <x:c r="B51" s="38"/>
       <x:c r="C51" s="39"/>
       <x:c r="D51" s="38"/>
-      <x:c r="E51" s="39"/>
-      <x:c r="F51" s="38"/>
-      <x:c r="G51" s="40"/>
+      <x:c r="E51" s="38"/>
+      <x:c r="F51" s="39"/>
+      <x:c r="G51" s="38"/>
       <x:c r="H51" s="40"/>
       <x:c r="I51" s="40"/>
       <x:c r="J51" s="40"/>
-      <x:c r="K51" s="39"/>
-      <x:c r="L51" s="41"/>
+      <x:c r="K51" s="40"/>
+      <x:c r="L51" s="39"/>
+      <x:c r="M51" s="41"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="E2:E51">
+      <x:formula1>"1,2,3"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77cba90d7dc24c32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re91b25209700443a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1439,7 +1501,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B8" s="54" t="str">
-        <x:v>Enter Date of Birth and the two dates as real Excel dates, not free-form text.</x:v>
+        <x:v>Choose Unit 1, 2 or 3. The portal automatically inserts the approved Unit and Unit Address into the Canva placeholders.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1447,7 +1509,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B9" s="54" t="str">
-        <x:v>Enter Bonus Amount as a positive number. The amount in words is generated automatically.</x:v>
+        <x:v>Enter Date of Birth and the two dates as real Excel dates, not free-form text.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1455,14 +1517,22 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B10" s="54" t="str">
+        <x:v>Enter Bonus Amount as a positive number. The amount in words is generated automatically.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="54" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="54" t="str">
         <x:v>In the portal, select the accounting year, upload this file, and review every employee before sending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="57" t="str">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="57" t="str">
         <x:v>Password</x:v>
       </x:c>
-      <x:c r="B11" s="57" t="str">
+      <x:c r="B12" s="57" t="str">
         <x:v>First 4 letters of employee name in uppercase + four-digit birth year (example: SAMP1992).</x:v>
       </x:c>
     </x:row>

</xml_diff>